<commit_message>
Add shell steps and GROUP column so Excel AT tests can mix local commands with serial AT.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/3_Python/at_framework/testcases/AT_Testcases_Template.xlsx
+++ b/3_Python/at_framework/testcases/AT_Testcases_Template.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Config" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Steps" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Reference" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Config" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Steps" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -430,7 +430,7 @@
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="48" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -463,7 +463,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Serial port（執行時可用命令列覆寫）</t>
+          <t>Serial port（Windows: COM14；Ubuntu: /dev/ttyACM0）</t>
         </is>
       </c>
     </row>
@@ -589,144 +589,156 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N11"/>
+  <dimension ref="A1:P12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="27" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="32" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="32" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="17" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="17" customWidth="1" min="13" max="13"/>
     <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="31" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>enabled</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>GROUP</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>test_id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>step</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>enabled</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>cmd</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>cmd_type</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>expect_type</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>expect_value</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>expect_label</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>timeout</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>idle_timeout</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>wait_after</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>reconnect_after</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>run_on_failure</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>check_ttff</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>note</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>GNSS</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
           <t>TC_GNSS_XTRA_ColdStart</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="D2" t="n">
         <v>1</v>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>AT!ENTERCND="A710"</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
         <is>
           <t>contains</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
-      </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="n">
-        <v>5</v>
       </c>
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="n">
+        <v>5</v>
+      </c>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="n">
         <v>0</v>
       </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
       <c r="M2" t="inlineStr">
         <is>
           <t>N</t>
@@ -734,57 +746,67 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
           <t>進入 CND 模式</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>GNSS</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
           <t>TC_GNSS_XTRA_ColdStart</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="D3" t="n">
         <v>2</v>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>AT!GPSCLRASSIST=1,1,1,1,1</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
         <is>
           <t>contains</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
-      </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="n">
-        <v>10</v>
       </c>
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="n">
+        <v>10</v>
+      </c>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="n">
         <v>0</v>
       </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
       <c r="M3" t="inlineStr">
         <is>
           <t>N</t>
@@ -792,61 +814,71 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
           <t>清除 assist data</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>GNSS</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
           <t>TC_GNSS_XTRA_ColdStart</t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="D4" t="n">
         <v>3</v>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>AT!GPSXTRASTATUS?</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
         <is>
           <t>contains</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>1980</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="n">
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="n">
         <v>30</v>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="J4" t="n">
+      <c r="L4" t="n">
         <v>0</v>
       </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
       <c r="M4" t="inlineStr">
         <is>
           <t>N</t>
@@ -854,61 +886,71 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
           <t>XTRA 應為初始狀態</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>GNSS</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
           <t>TC_GNSS_XTRA_ColdStart</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="D5" t="n">
         <v>4</v>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>AT!GPSXTRAINITDNLD</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
         <is>
           <t>contains</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>Xtra command sent successfully</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="n">
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="n">
         <v>60</v>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="J5" t="n">
+      <c r="L5" t="n">
         <v>0</v>
       </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
       <c r="M5" t="inlineStr">
         <is>
           <t>N</t>
@@ -916,61 +958,71 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
           <t>觸發 XTRA 下載</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>GNSS</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
           <t>TC_GNSS_XTRA_ColdStart</t>
         </is>
       </c>
-      <c r="B6" t="n">
+      <c r="D6" t="n">
         <v>5</v>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>AT!GPSXTRASTATUS?</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
         <is>
           <t>custom</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>current_year_month</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="n">
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="n">
         <v>30</v>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="J6" t="n">
+      <c r="L6" t="n">
         <v>0</v>
       </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
       <c r="M6" t="inlineStr">
         <is>
           <t>N</t>
@@ -978,57 +1030,67 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
           <t>XTRA 日期應為今年今月</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>GNSS</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
           <t>TC_GNSS_XTRA_ColdStart</t>
         </is>
       </c>
-      <c r="B7" t="n">
+      <c r="D7" t="n">
         <v>6</v>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>AT!GPSFIX=1,255,255</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
         <is>
           <t>contains</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
-      </c>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="n">
-        <v>30</v>
       </c>
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="n">
+        <v>30</v>
+      </c>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="n">
         <v>5</v>
       </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
       <c r="M7" t="inlineStr">
         <is>
           <t>N</t>
@@ -1036,177 +1098,207 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
           <t>Cold start fix</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>GNSS</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
           <t>TC_GNSS_XTRA_ColdStart</t>
         </is>
       </c>
-      <c r="B8" t="n">
+      <c r="D8" t="n">
         <v>7</v>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>AT!GPSSTATUS?</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>custom</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>gps_status_ttff</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="n">
+        <v>30</v>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="L8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>檢查 TTFF</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
         <is>
           <t>V</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>AT!GPSSTATUS?</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>custom</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>gps_status_ttff</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="n">
-        <v>30</v>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="J8" t="n">
-        <v>0</v>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>檢查 TTFF</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>GNSS</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
           <t>TC_GNSS_XTRA_ColdStart</t>
         </is>
       </c>
-      <c r="B9" t="n">
+      <c r="D9" t="n">
         <v>8</v>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>AT!GPSEND=0</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
         <is>
           <t>contains</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="H9" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
-      </c>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="n">
-        <v>10</v>
       </c>
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="n">
+        <v>10</v>
+      </c>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="n">
         <v>0</v>
       </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L9" t="inlineStr">
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
         <is>
           <t>V</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="N9" t="inlineStr">
+      <c r="O9" t="inlineStr">
         <is>
           <t>收尾；失敗時仍執行</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Smoke</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
           <t>TC_Smoke_AT</t>
         </is>
       </c>
-      <c r="B10" t="n">
+      <c r="D10" t="n">
         <v>1</v>
       </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>AT</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
         <is>
           <t>contains</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="H10" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
-      </c>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="n">
-        <v>2</v>
       </c>
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="n">
+        <v>2</v>
+      </c>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="n">
         <v>0</v>
       </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
       <c r="M10" t="inlineStr">
         <is>
           <t>N</t>
@@ -1214,57 +1306,67 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
           <t>基本握手</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Smoke</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
           <t>TC_Smoke_AT</t>
         </is>
       </c>
-      <c r="B11" t="n">
+      <c r="D11" t="n">
         <v>2</v>
       </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>ATI</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
         <is>
           <t>regex</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="H11" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
-      </c>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="n">
-        <v>2</v>
       </c>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="n">
+        <v>2</v>
+      </c>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="n">
         <v>0</v>
       </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
       <c r="M11" t="inlineStr">
         <is>
           <t>N</t>
@@ -1272,7 +1374,85 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
           <t>查詢版本</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Shell</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>TC_Shell_Smoke</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>echo at_framework_shell_ok</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>shell</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>contains</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>at_framework_shell_ok</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="n">
+        <v>5</v>
+      </c>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>本機 shell 煙霧測試；可單獨 -t 執行、不必接模組</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>N</t>
         </is>
       </c>
     </row>
@@ -1287,11 +1467,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
     <col width="25" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
@@ -1315,216 +1495,216 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>test_id</t>
+          <t>enabled</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>測試案例 ID，同 ID 多列組成一個序列</t>
+          <t>A 欄。V=執行 / N=略過</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>TC_GNSS_XTRA_ColdStart</t>
+          <t>V</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>step</t>
+          <t>GROUP</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>步驟順序（整數）</t>
+          <t>B 欄。分類標籤（執行時不影響；可空）</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>GNSS</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>enabled</t>
+          <t>test_id</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>V=執行 / N=略過</t>
+          <t>C 欄。測試案例 ID，同 ID 多列組成一個序列</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>TC_GNSS_XTRA_ColdStart</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>cmd</t>
+          <t>step</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>AT 指令（不含 \r\n）</t>
+          <t>D 欄。步驟順序（整數）</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>expect_type</t>
+          <t>cmd</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>contains | regex | custom</t>
+          <t>E 欄。AT 或 shell 指令（AT 不含 \r\n；簡訊本文結尾寫 {CTRLZ}）</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>contains</t>
+          <t>Test SMS{CTRLZ}</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>expect_value</t>
+          <t>cmd_type</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>預期內容或 custom 名稱</t>
+          <t>F 欄。空白或 at=經 serial 送 AT；shell=本機（Ubuntu bash）執行</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>OK / current_year_month</t>
+          <t>at / shell</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>expect_label</t>
+          <t>expect_type</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>報告顯示用（可空）</t>
+          <t>G 欄。contains | regex | custom</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>TTFF (sec) &lt; 5</t>
+          <t>contains</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>timeout</t>
+          <t>expect_value</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>此步驟最長等待秒數</t>
+          <t>H 欄。預期內容或 custom 名稱</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>OK / current_year_month</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>idle_timeout</t>
+          <t>expect_label</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>空=0.3；none=等到 timeout</t>
+          <t>I 欄。報告顯示用（可空）</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>TTFF (sec) &lt; 5</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>wait_after</t>
+          <t>timeout</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>本步驟完成後等待秒數</t>
+          <t>J 欄。此步驟最長等待秒數</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>30</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>reconnect_after</t>
+          <t>idle_timeout</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>V=等待後關閉並重連 serial（模組會重啟時用）</t>
+          <t>K 欄。空=0.3；none=等到 timeout</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>none</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>run_on_failure</t>
+          <t>wait_after</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>V=前步失敗時仍執行此步</t>
+          <t>L 欄。本步驟完成後等待秒數</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>5</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>check_ttff</t>
+          <t>reconnect_after</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>V=額外寫 TTFF 判定 log</t>
+          <t>M 欄。V=等待後關閉並重連 serial（模組會重啟時用）</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1536,56 +1716,64 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>run_on_failure</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>N 欄。V=前步失敗時仍執行此步</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
           <t>note</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>備註</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr"/>
-      <c r="B16" t="inlineStr"/>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>O 欄。備註</t>
+        </is>
+      </c>
       <c r="C16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>custom 名稱</t>
+          <t>check_ttff</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>說明</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr"/>
+          <t>P 欄。V=額外寫 TTFF 判定 log</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>current_year_month</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>回應含今年+空格+兩位數月份</t>
-        </is>
-      </c>
+      <c r="A18" t="inlineStr"/>
+      <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>gps_status_ttff</t>
+          <t>custom 名稱</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>OK 且 TTFF &lt; 5</t>
+          <t>說明</t>
         </is>
       </c>
       <c r="C19" t="inlineStr"/>
@@ -1593,15 +1781,41 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
+          <t>current_year_month</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>回應含今年+空格+兩位數月份</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>gps_status_ttff</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>OK 且 TTFF &lt; 5</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
           <t>gps_status_ttff:3</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B22" t="inlineStr">
         <is>
           <t>OK 且 TTFF &lt; 3</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr"/>
+      <c r="C22" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>